<commit_message>
updated file made in january. will remove soon
</commit_message>
<xml_diff>
--- a/data/FY2025 Files/summary_file_FY2025_2026-01-23.xlsx
+++ b/data/FY2025 Files/summary_file_FY2025_2026-01-23.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aleaw\Documents\PhD Fall 2021 - Spring 2022\Merriman RA\Fiscal Futures IGPA\Fiscal-Future-Topics\data\FY2025 Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2F073F1-F506-44D1-B488-9413D809A798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F9FC11F-55DA-4916-8201-65ABCF565227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10455" yWindow="-16200" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10455" yWindow="-16200" windowWidth="14400" windowHeight="7800" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="aggregated_totals_long" sheetId="8" r:id="rId1"/>
@@ -897,7 +897,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="170" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -923,13 +934,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -32977,6 +32991,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D29"/>
   <sheetFormatPr defaultColWidth="10.9453125" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="2" max="3" width="13.20703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.7890625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
@@ -32996,13 +33014,13 @@
       <c r="A2">
         <v>1998</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>31241.142268420001</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="1">
         <v>32028.331688760001</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="1">
         <v>787.18942034000099</v>
       </c>
     </row>
@@ -33010,13 +33028,13 @@
       <c r="A3">
         <v>1999</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>33845.350926309999</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="1">
         <v>33963.525296760003</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="1">
         <v>118.17437045000401</v>
       </c>
     </row>
@@ -33024,13 +33042,13 @@
       <c r="A4">
         <v>2000</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>37340.660437159997</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="1">
         <v>37041.391645399999</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="1">
         <v>-299.26879175999801</v>
       </c>
     </row>
@@ -33038,13 +33056,13 @@
       <c r="A5">
         <v>2001</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <v>40354.009028469998</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="1">
         <v>38278.700592430003</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="1">
         <v>-2075.3084360399998</v>
       </c>
     </row>
@@ -33052,13 +33070,13 @@
       <c r="A6">
         <v>2002</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="1">
         <v>42063.830838349997</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="1">
         <v>37919.379338059996</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="1">
         <v>-4144.4515002899998</v>
       </c>
     </row>
@@ -33066,13 +33084,13 @@
       <c r="A7">
         <v>2003</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="1">
         <v>42608.364008709999</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="1">
         <v>38449.20157148</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="1">
         <v>-4159.1624372300003</v>
       </c>
     </row>
@@ -33080,13 +33098,13 @@
       <c r="A8">
         <v>2004</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="1">
         <v>53019.315220620003</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="1">
         <v>42605.136041489997</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="1">
         <v>-10414.17917913</v>
       </c>
     </row>
@@ -33094,13 +33112,13 @@
       <c r="A9">
         <v>2005</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="1">
         <v>45358.950389769998</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="1">
         <v>44301.935573369999</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="1">
         <v>-1057.0148164</v>
       </c>
     </row>
@@ -33108,13 +33126,13 @@
       <c r="A10">
         <v>2006</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="1">
         <v>48059.471020739998</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="1">
         <v>46165.60639026</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="1">
         <v>-1893.86463048</v>
       </c>
     </row>
@@ -33122,13 +33140,13 @@
       <c r="A11">
         <v>2007</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="1">
         <v>51127.60051199</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="1">
         <v>49489.71073287</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="1">
         <v>-1637.88977912</v>
       </c>
     </row>
@@ -33136,13 +33154,13 @@
       <c r="A12">
         <v>2008</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="1">
         <v>54169.864453100003</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="1">
         <v>51636.908789779998</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="1">
         <v>-2532.95566332</v>
       </c>
     </row>
@@ -33150,13 +33168,13 @@
       <c r="A13">
         <v>2009</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="1">
         <v>56749.683344309997</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="1">
         <v>51460.958706819998</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="1">
         <v>-5288.7246374899996</v>
       </c>
     </row>
@@ -33164,13 +33182,13 @@
       <c r="A14">
         <v>2010</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="1">
         <v>58047.799746309996</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="1">
         <v>51191.541425249998</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="1">
         <v>-6856.2583210599996</v>
       </c>
     </row>
@@ -33178,13 +33196,13 @@
       <c r="A15">
         <v>2011</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="1">
         <v>58419.425721690001</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="1">
         <v>56299.281941729998</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="1">
         <v>-2120.1437799599998</v>
       </c>
     </row>
@@ -33192,13 +33210,13 @@
       <c r="A16">
         <v>2012</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="1">
         <v>59861.24594565</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="1">
         <v>58417.847561850002</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="1">
         <v>-1443.3983837999999</v>
       </c>
     </row>
@@ -33206,13 +33224,13 @@
       <c r="A17">
         <v>2013</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="1">
         <v>63284.886307699999</v>
       </c>
-      <c r="C17">
+      <c r="C17" s="1">
         <v>63096.99085794</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="1">
         <v>-187.895449759999</v>
       </c>
     </row>
@@ -33220,13 +33238,13 @@
       <c r="A18">
         <v>2014</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="1">
         <v>66962.793097689995</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="1">
         <v>65263.785644900003</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="1">
         <v>-1699.0074527899901</v>
       </c>
     </row>
@@ -33234,13 +33252,13 @@
       <c r="A19">
         <v>2015</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="1">
         <v>69937.376507930006</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="1">
         <v>66584.603653209997</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="1">
         <v>-3352.7728547200099</v>
       </c>
     </row>
@@ -33248,13 +33266,13 @@
       <c r="A20">
         <v>2016</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="1">
         <v>63928.130405210002</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="1">
         <v>64148.84226677</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="1">
         <v>220.711861559997</v>
       </c>
     </row>
@@ -33262,13 +33280,13 @@
       <c r="A21">
         <v>2017</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="1">
         <v>71724.190436100005</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="1">
         <v>63653.854908840003</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="1">
         <v>-8070.3355272600002</v>
       </c>
     </row>
@@ -33276,13 +33294,13 @@
       <c r="A22">
         <v>2018</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="1">
         <v>74966.127536920001</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="1">
         <v>73008.551489699996</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="1">
         <v>-1957.57604722001</v>
       </c>
     </row>
@@ -33290,13 +33308,13 @@
       <c r="A23">
         <v>2019</v>
       </c>
-      <c r="B23">
+      <c r="B23" s="1">
         <v>74401.846659190007</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="1">
         <v>74631.657433760003</v>
       </c>
-      <c r="D23">
+      <c r="D23" s="1">
         <v>229.810774569996</v>
       </c>
     </row>
@@ -33304,13 +33322,13 @@
       <c r="A24">
         <v>2020</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="1">
         <v>81603.22934659</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="1">
         <v>80582.050002880002</v>
       </c>
-      <c r="D24">
+      <c r="D24" s="1">
         <v>-1021.17934371</v>
       </c>
     </row>
@@ -33318,13 +33336,13 @@
       <c r="A25">
         <v>2021</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="1">
         <v>92883.163981389996</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="1">
         <v>95200.508864670002</v>
       </c>
-      <c r="D25">
+      <c r="D25" s="1">
         <v>2317.34488328001</v>
       </c>
     </row>
@@ -33332,13 +33350,13 @@
       <c r="A26">
         <v>2022</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="1">
         <v>100065.05532539</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="1">
         <v>116055.6865928</v>
       </c>
-      <c r="D26">
+      <c r="D26" s="1">
         <v>15990.631267410001</v>
       </c>
     </row>
@@ -33346,13 +33364,13 @@
       <c r="A27">
         <v>2023</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="1">
         <v>111971.76886872</v>
       </c>
-      <c r="C27">
+      <c r="C27" s="1">
         <v>111766.06624185</v>
       </c>
-      <c r="D27">
+      <c r="D27" s="1">
         <v>-205.70262686999899</v>
       </c>
     </row>
@@ -33360,13 +33378,13 @@
       <c r="A28">
         <v>2024</v>
       </c>
-      <c r="B28">
+      <c r="B28" s="1">
         <v>114997.03737177</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="1">
         <v>115121.08453568</v>
       </c>
-      <c r="D28">
+      <c r="D28" s="1">
         <v>124.04716390999999</v>
       </c>
     </row>
@@ -33374,13 +33392,13 @@
       <c r="A29">
         <v>2025</v>
       </c>
-      <c r="B29">
+      <c r="B29" s="1">
         <v>119505.48449939</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="1">
         <v>118157.29579629999</v>
       </c>
-      <c r="D29">
+      <c r="D29" s="1">
         <v>-1348.18870309001</v>
       </c>
     </row>

</xml_diff>